<commit_message>
Correct weekly topics and restore branding
Restore the complete how-it-works content, preserve multiple topic headings per week through Excel import and export, regenerate the canonical workbooks, and use the original TWB logo across shared branding.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>

Copilot-Session: dc045078-7d35-4ca3-b3d0-dad33d481668
</commit_message>
<xml_diff>
--- a/konusma-konulari-sablon.xlsx
+++ b/konusma-konulari-sablon.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Hafta 1 - Friendship" sheetId="1" r:id="rId1"/>
-    <sheet name="Hafta 2 - Travel" sheetId="2" r:id="rId2"/>
+    <sheet name="Hafta 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hafta 2" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -398,11 +398,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:B5"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="78.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -410,9 +409,6 @@
         <v>Başlık</v>
       </c>
       <c r="B1" t="str">
-        <v>Kategori</v>
-      </c>
-      <c r="C1" t="str">
         <v>Soru</v>
       </c>
     </row>
@@ -421,37 +417,46 @@
         <v>Friendship</v>
       </c>
       <c r="B2" t="str">
-        <v>Warm-up</v>
-      </c>
-      <c r="C2" t="str">
         <v>What makes someone a good friend?</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Friendship</v>
+        <v/>
       </c>
       <c r="B3" t="str">
-        <v>Discussion</v>
-      </c>
-      <c r="C3" t="str">
         <v>How do friendships change as we grow older?</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Trust</v>
+      </c>
+      <c r="B4" t="str">
+        <v>How can a person earn another person's trust?</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v>Why is trust important in a friendship?</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:B3"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="78.83203125" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,9 +464,6 @@
         <v>Başlık</v>
       </c>
       <c r="B1" t="str">
-        <v>Kategori</v>
-      </c>
-      <c r="C1" t="str">
         <v>Soru</v>
       </c>
     </row>
@@ -470,15 +472,20 @@
         <v>Travel</v>
       </c>
       <c r="B2" t="str">
-        <v>Warm-up</v>
-      </c>
-      <c r="C2" t="str">
         <v>Where would you most like to travel?</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v>What can people learn by visiting another country?</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>